<commit_message>
Add CEO field, allow negative other costs, restyle inputs
- Add a 대표이사 input next to the company name (exported to H5)
- Rename 기타 잡비 to 기타 비용 and accept negative values there
- Pick up workbook changes: labor cost formula, Tqoon fee on gross sales,
  new defaults
- Blue inputs, red negatives, narrower layout, right-aligned exchange rate

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BusinessPlan.xlsx
+++ b/BusinessPlan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TS LEE\Documents\TQBusinessPlan_AI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EC32B42-9E43-4BE8-8C79-DE0B9D1C1AFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9257A46C-CDDE-4C1C-A1C7-61214509D4C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{7FB24EEC-24BD-434D-87DD-9AB09F683891}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="54">
   <si>
     <t>준비</t>
   </si>
@@ -220,6 +220,9 @@
   <si>
     <t>* 인건비 = 급여+상여금(200%)+퇴직적립금(100%)+국민연금(4.75%)+건강보험(3.595%)+장기요양보험(건강보험의 13.14%)+고용보험 (1.15%)</t>
   </si>
+  <si>
+    <t>대표이사 명:</t>
+  </si>
 </sst>
 </file>
 
@@ -231,7 +234,7 @@
     <numFmt numFmtId="165" formatCode="\(#,##0\);\(\-#,##0\)"/>
     <numFmt numFmtId="166" formatCode="#,##0_ ;\-#,##0\ "/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -309,6 +312,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -525,7 +535,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -611,6 +621,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1022,7 +1035,9 @@
       </c>
       <c r="E5" s="40"/>
       <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
+      <c r="G5" s="53" t="s">
+        <v>53</v>
+      </c>
       <c r="H5" s="41"/>
       <c r="I5" s="41"/>
       <c r="J5" s="41"/>
@@ -1372,30 +1387,30 @@
         <v>37</v>
       </c>
       <c r="F25" s="42">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="G25" s="12" t="s">
         <v>36</v>
       </c>
       <c r="H25" s="24">
         <f>F25*12</f>
-        <v>12000000</v>
+        <v>6000000</v>
       </c>
       <c r="I25" s="24">
         <f>H25*1.03</f>
-        <v>12360000</v>
+        <v>6180000</v>
       </c>
       <c r="J25" s="24">
         <f t="shared" ref="J25" si="2">I25*1.03</f>
-        <v>12730800</v>
+        <v>6365400</v>
       </c>
       <c r="K25" s="24">
         <f t="shared" ref="K25" si="3">J25*1.03</f>
-        <v>13112724</v>
+        <v>6556362</v>
       </c>
       <c r="L25" s="24">
         <f>K25*1.03</f>
-        <v>13506105.720000001</v>
+        <v>6753052.8600000003</v>
       </c>
       <c r="M25" s="11"/>
     </row>
@@ -1646,28 +1661,28 @@
       </c>
       <c r="F33" s="14">
         <f>SUM(F24:F32)</f>
-        <v>8500000.0500000007</v>
+        <v>8000000.0499999998</v>
       </c>
       <c r="G33" s="12"/>
       <c r="H33" s="24">
         <f>SUM(H24:H32)</f>
-        <v>126736900</v>
+        <v>120736900</v>
       </c>
       <c r="I33" s="24">
         <f>SUM(I24:I32)</f>
-        <v>141424207</v>
+        <v>135244207</v>
       </c>
       <c r="J33" s="24">
         <f>SUM(J24:J32)</f>
-        <v>150700933.21000001</v>
+        <v>144335533.21000001</v>
       </c>
       <c r="K33" s="24">
         <f>SUM(K24:K32)</f>
-        <v>157330361.20630002</v>
+        <v>150773999.20630002</v>
       </c>
       <c r="L33" s="24">
         <f>SUM(L24:L32)</f>
-        <v>164075872.04248902</v>
+        <v>157322819.18248904</v>
       </c>
       <c r="M33" s="11"/>
     </row>
@@ -1993,23 +2008,23 @@
       <c r="G47" s="12"/>
       <c r="H47" s="24">
         <f>H33+H44</f>
-        <v>161512900</v>
+        <v>155512900</v>
       </c>
       <c r="I47" s="24">
         <f>I33+I44</f>
-        <v>315304207</v>
+        <v>309124207</v>
       </c>
       <c r="J47" s="24">
         <f>J33+J44</f>
-        <v>394132933.20999998</v>
+        <v>387767533.20999998</v>
       </c>
       <c r="K47" s="24">
         <f>K33+K44</f>
-        <v>435538361.20630002</v>
+        <v>428981999.20630002</v>
       </c>
       <c r="L47" s="24">
         <f>L33+L44</f>
-        <v>477059872.04248905</v>
+        <v>470306819.18248904</v>
       </c>
       <c r="M47" s="11"/>
     </row>
@@ -2037,23 +2052,23 @@
       </c>
       <c r="H49" s="46">
         <f t="shared" si="12"/>
-        <v>-106312900</v>
+        <v>-100312900</v>
       </c>
       <c r="I49" s="46">
         <f t="shared" si="12"/>
-        <v>-39304207</v>
+        <v>-33124207</v>
       </c>
       <c r="J49" s="46">
         <f t="shared" si="12"/>
-        <v>-7732933.2100000381</v>
+        <v>-1367533.2100000381</v>
       </c>
       <c r="K49" s="46">
         <f t="shared" si="12"/>
-        <v>6061638.7936999798</v>
+        <v>12618000.79369998</v>
       </c>
       <c r="L49" s="46">
         <f t="shared" si="12"/>
-        <v>19740127.957510948</v>
+        <v>26493180.817510962</v>
       </c>
       <c r="M49" s="11"/>
     </row>
@@ -2069,23 +2084,23 @@
       </c>
       <c r="H50" s="27">
         <f>G50+H49</f>
-        <v>-136312900</v>
+        <v>-130312900</v>
       </c>
       <c r="I50" s="27">
         <f>H50+I49</f>
-        <v>-175617107</v>
+        <v>-163437107</v>
       </c>
       <c r="J50" s="27">
         <f t="shared" ref="J50:L50" si="13">I50+J49</f>
-        <v>-183350040.21000004</v>
+        <v>-164804640.21000004</v>
       </c>
       <c r="K50" s="27">
         <f t="shared" si="13"/>
-        <v>-177288401.41630006</v>
+        <v>-152186639.41630006</v>
       </c>
       <c r="L50" s="27">
         <f t="shared" si="13"/>
-        <v>-157548273.45878911</v>
+        <v>-125693458.5987891</v>
       </c>
       <c r="M50" s="11"/>
     </row>
@@ -2113,23 +2128,23 @@
       </c>
       <c r="H52" s="35">
         <f t="shared" si="14"/>
-        <v>63687100</v>
+        <v>69687100</v>
       </c>
       <c r="I52" s="35">
         <f t="shared" si="14"/>
-        <v>24382893</v>
+        <v>36562893</v>
       </c>
       <c r="J52" s="35">
         <f t="shared" si="14"/>
-        <v>16649959.789999962</v>
+        <v>35195359.789999962</v>
       </c>
       <c r="K52" s="35">
         <f t="shared" si="14"/>
-        <v>22711598.583699942</v>
+        <v>47813360.583699942</v>
       </c>
       <c r="L52" s="35">
         <f t="shared" si="14"/>
-        <v>42451726.54121089</v>
+        <v>74306541.401210904</v>
       </c>
       <c r="M52" s="11"/>
     </row>

</xml_diff>

<commit_message>
Sync web calculator with revised workbook
- Add 사무실 임대 보증금 to initial costs; rows below shift down by one
- Profit/loss is now sales minus costs; cash starts at investment minus
  initial costs and accumulates yearly profit
- Read blue bold numbers as the input cells, matching the workbook
- New defaults for rent, yen sales, logistics and customs rates

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BusinessPlan.xlsx
+++ b/BusinessPlan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TS LEE\Documents\TQBusinessPlan_AI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9257A46C-CDDE-4C1C-A1C7-61214509D4C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A259E456-FAD2-4852-AE59-DB14FB13F040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{7FB24EEC-24BD-434D-87DD-9AB09F683891}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="55">
   <si>
     <t>준비</t>
   </si>
@@ -174,9 +174,6 @@
   </si>
   <si>
     <t>접대비/복리후생비</t>
-  </si>
-  <si>
-    <t>기타 잡비</t>
   </si>
   <si>
     <r>
@@ -223,18 +220,25 @@
   <si>
     <t>대표이사 명:</t>
   </si>
+  <si>
+    <t>기타 비용</t>
+  </si>
+  <si>
+    <t>사무실 임대 보증금</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="\(#,##0\);\(#,##0\)"/>
-    <numFmt numFmtId="165" formatCode="\(#,##0\);\(\-#,##0\)"/>
     <numFmt numFmtId="166" formatCode="#,##0_ ;\-#,##0\ "/>
+    <numFmt numFmtId="167" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
+    <numFmt numFmtId="168" formatCode="\(#,##0\);[Red]\(\-#,##0\)"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -319,6 +323,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -535,7 +547,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -568,7 +580,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -579,7 +590,6 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
@@ -600,18 +610,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="2" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -620,12 +619,24 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="41" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="41" fontId="11" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="41" fontId="11" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="쉼표 [0]" xfId="1" builtinId="6"/>
@@ -961,12 +972,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFBDFD68-C366-4AFA-AA68-57F3CCAF5EEC}">
-  <dimension ref="B1:M53"/>
+  <dimension ref="B1:M54"/>
   <sheetFormatPr defaultRowHeight="14.65" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="1.29296875" customWidth="1"/>
-    <col min="3" max="3" width="10.5859375" style="23" customWidth="1"/>
+    <col min="3" max="3" width="10.5859375" style="22" customWidth="1"/>
     <col min="4" max="4" width="10.17578125" customWidth="1"/>
     <col min="5" max="5" width="18.41015625" customWidth="1"/>
     <col min="6" max="6" width="11.41015625" style="1" customWidth="1"/>
@@ -981,7 +992,7 @@
     <row r="1" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:13" ht="6.6" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B2" s="6"/>
-      <c r="C2" s="29"/>
+      <c r="C2" s="27"/>
       <c r="D2" s="7"/>
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
@@ -995,19 +1006,19 @@
     </row>
     <row r="3" spans="2:13" ht="21" x14ac:dyDescent="0.65">
       <c r="B3" s="10"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="50" t="s">
+      <c r="C3" s="28"/>
+      <c r="D3" s="41" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="51"/>
-      <c r="F3" s="52" t="s">
+      <c r="E3" s="42"/>
+      <c r="F3" s="50" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="52"/>
-      <c r="J3" s="52"/>
-      <c r="K3" s="52"/>
+      <c r="G3" s="50"/>
+      <c r="H3" s="50"/>
+      <c r="I3" s="50"/>
+      <c r="J3" s="50"/>
+      <c r="K3" s="50"/>
       <c r="L3" s="1" t="s">
         <v>22</v>
       </c>
@@ -1015,64 +1026,64 @@
     </row>
     <row r="4" spans="2:13" ht="7.5" customHeight="1" x14ac:dyDescent="0.65">
       <c r="B4" s="10"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
-      <c r="I4" s="41"/>
-      <c r="J4" s="41"/>
-      <c r="K4" s="41"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="39"/>
+      <c r="G4" s="39"/>
+      <c r="H4" s="39"/>
+      <c r="I4" s="39"/>
+      <c r="J4" s="39"/>
+      <c r="K4" s="39"/>
       <c r="L4" s="1"/>
       <c r="M4" s="11"/>
     </row>
     <row r="5" spans="2:13" ht="21" x14ac:dyDescent="0.65">
       <c r="B5" s="10"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="E5" s="40"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="53" t="s">
-        <v>53</v>
-      </c>
-      <c r="H5" s="41"/>
-      <c r="I5" s="41"/>
-      <c r="J5" s="41"/>
-      <c r="K5" s="41"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="38"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="H5" s="39"/>
+      <c r="I5" s="39"/>
+      <c r="J5" s="39"/>
+      <c r="K5" s="39"/>
       <c r="L5" s="1"/>
       <c r="M5" s="11"/>
     </row>
     <row r="6" spans="2:13" ht="21" x14ac:dyDescent="0.65">
       <c r="B6" s="10"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="E6" s="40"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="41"/>
-      <c r="I6" s="41"/>
-      <c r="J6" s="41"/>
-      <c r="K6" s="41"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="22" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="38"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="39"/>
+      <c r="H6" s="39"/>
+      <c r="I6" s="39"/>
+      <c r="J6" s="39"/>
+      <c r="K6" s="39"/>
       <c r="L6" s="1"/>
       <c r="M6" s="11"/>
     </row>
     <row r="7" spans="2:13" ht="12.6" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B7" s="10"/>
-      <c r="C7" s="30"/>
+      <c r="C7" s="28"/>
       <c r="M7" s="11"/>
     </row>
     <row r="8" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B8" s="10"/>
-      <c r="C8" s="30"/>
-      <c r="E8" s="49" t="s">
+      <c r="C8" s="28"/>
+      <c r="E8" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="F8" s="49"/>
+      <c r="F8" s="45"/>
       <c r="G8" s="5" t="s">
         <v>0</v>
       </c>
@@ -1095,11 +1106,11 @@
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B9" s="10"/>
-      <c r="C9" s="30"/>
+      <c r="C9" s="28"/>
       <c r="D9" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="47">
+      <c r="E9" s="49">
         <v>9.1999999999999993</v>
       </c>
       <c r="F9" s="1" t="s">
@@ -1115,7 +1126,7 @@
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B10" s="10"/>
-      <c r="C10" s="30"/>
+      <c r="C10" s="28"/>
       <c r="G10" s="12"/>
       <c r="H10" s="12"/>
       <c r="I10" s="12"/>
@@ -1126,10 +1137,10 @@
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B11" s="10"/>
-      <c r="C11" s="38" t="s">
-        <v>46</v>
-      </c>
-      <c r="G11" s="42">
+      <c r="C11" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" s="43">
         <v>200000000</v>
       </c>
       <c r="H11" s="12"/>
@@ -1141,7 +1152,7 @@
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B12" s="10"/>
-      <c r="C12" s="30"/>
+      <c r="C12" s="28"/>
       <c r="G12" s="13"/>
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
@@ -1152,14 +1163,14 @@
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B13" s="10"/>
-      <c r="C13" s="30"/>
+      <c r="C13" s="28"/>
       <c r="D13" t="s">
         <v>27</v>
       </c>
       <c r="E13" t="s">
         <v>25</v>
       </c>
-      <c r="G13" s="37">
+      <c r="G13" s="35">
         <v>2000000</v>
       </c>
       <c r="H13" s="12"/>
@@ -1171,11 +1182,11 @@
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B14" s="10"/>
-      <c r="C14" s="30"/>
+      <c r="C14" s="28"/>
       <c r="E14" t="s">
         <v>24</v>
       </c>
-      <c r="G14" s="42">
+      <c r="G14" s="43">
         <v>2000000</v>
       </c>
       <c r="H14" s="12"/>
@@ -1187,11 +1198,11 @@
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B15" s="10"/>
-      <c r="C15" s="30"/>
+      <c r="C15" s="28"/>
       <c r="E15" t="s">
         <v>1</v>
       </c>
-      <c r="G15" s="42">
+      <c r="G15" s="43">
         <v>15000000</v>
       </c>
       <c r="H15" s="12"/>
@@ -1203,11 +1214,11 @@
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B16" s="10"/>
-      <c r="C16" s="30"/>
+      <c r="C16" s="28"/>
       <c r="E16" t="s">
-        <v>3</v>
-      </c>
-      <c r="G16" s="42">
+        <v>54</v>
+      </c>
+      <c r="G16" s="43">
         <v>10000000</v>
       </c>
       <c r="H16" s="12"/>
@@ -1219,13 +1230,12 @@
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B17" s="10"/>
-      <c r="C17" s="30"/>
-      <c r="E17" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F17" s="3"/>
-      <c r="G17" s="48">
-        <v>1000000</v>
+      <c r="C17" s="28"/>
+      <c r="E17" t="s">
+        <v>3</v>
+      </c>
+      <c r="G17" s="43">
+        <v>10000000</v>
       </c>
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
@@ -1236,13 +1246,13 @@
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B18" s="10"/>
-      <c r="C18" s="30"/>
-      <c r="E18" t="s">
-        <v>7</v>
-      </c>
-      <c r="G18" s="12">
-        <f>SUM(G13:G17)</f>
-        <v>30000000</v>
+      <c r="C18" s="28"/>
+      <c r="E18" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F18" s="3"/>
+      <c r="G18" s="44">
+        <v>1000000</v>
       </c>
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
@@ -1253,914 +1263,925 @@
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B19" s="10"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
+      <c r="C19" s="28"/>
+      <c r="E19" t="s">
+        <v>7</v>
+      </c>
+      <c r="G19" s="12">
+        <f>SUM(G13:G18)</f>
+        <v>40000000</v>
+      </c>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="12"/>
       <c r="M19" s="11"/>
     </row>
-    <row r="20" spans="2:13" ht="4.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B20" s="10"/>
-      <c r="C20" s="30"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="12"/>
-      <c r="L20" s="12"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
       <c r="M20" s="11"/>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:13" ht="4.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B21" s="10"/>
-      <c r="C21" s="30" t="s">
+      <c r="C21" s="28"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="12"/>
+      <c r="M21" s="11"/>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B22" s="10"/>
+      <c r="C22" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="G21" s="12"/>
-      <c r="H21" s="24">
-        <f>H22*$E$9*12</f>
+      <c r="G22" s="12"/>
+      <c r="H22" s="23">
+        <f>H23*$E$9*12</f>
         <v>55200000</v>
       </c>
-      <c r="I21" s="24">
-        <f t="shared" ref="I21:L21" si="0">I22*$E$9*12</f>
+      <c r="I22" s="23">
+        <f t="shared" ref="I22:L22" si="0">I23*$E$9*12</f>
         <v>276000000</v>
       </c>
-      <c r="J21" s="24">
+      <c r="J22" s="23">
+        <f t="shared" si="0"/>
+        <v>331199999.99999994</v>
+      </c>
+      <c r="K22" s="23">
         <f t="shared" si="0"/>
         <v>386399999.99999994</v>
       </c>
-      <c r="K21" s="24">
+      <c r="L22" s="23">
         <f t="shared" si="0"/>
         <v>441600000</v>
       </c>
-      <c r="L21" s="24">
-        <f t="shared" si="0"/>
-        <v>496800000</v>
-      </c>
-      <c r="M21" s="11"/>
-    </row>
-    <row r="22" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B22" s="10"/>
-      <c r="C22" s="30"/>
-      <c r="E22" t="s">
-        <v>50</v>
-      </c>
-      <c r="G22" t="s">
-        <v>35</v>
-      </c>
-      <c r="H22" s="45">
-        <v>500000</v>
-      </c>
-      <c r="I22" s="45">
-        <v>2500000</v>
-      </c>
-      <c r="J22" s="45">
-        <v>3500000</v>
-      </c>
-      <c r="K22" s="45">
-        <v>4000000</v>
-      </c>
-      <c r="L22" s="45">
-        <v>4500000</v>
-      </c>
       <c r="M22" s="11"/>
     </row>
     <row r="23" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B23" s="10"/>
-      <c r="C23" s="30"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="24"/>
-      <c r="I23" s="24"/>
-      <c r="J23" s="24"/>
-      <c r="K23" s="24"/>
-      <c r="L23" s="24"/>
+      <c r="C23" s="28"/>
+      <c r="E23" t="s">
+        <v>49</v>
+      </c>
+      <c r="G23" t="s">
+        <v>35</v>
+      </c>
+      <c r="H23" s="48">
+        <v>500000</v>
+      </c>
+      <c r="I23" s="48">
+        <v>2500000</v>
+      </c>
+      <c r="J23" s="48">
+        <v>3000000</v>
+      </c>
+      <c r="K23" s="48">
+        <v>3500000</v>
+      </c>
+      <c r="L23" s="48">
+        <v>4000000</v>
+      </c>
       <c r="M23" s="11"/>
     </row>
     <row r="24" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B24" s="10"/>
-      <c r="C24" s="30" t="s">
-        <v>12</v>
-      </c>
-      <c r="D24" t="s">
-        <v>40</v>
-      </c>
-      <c r="E24" t="s">
-        <v>43</v>
-      </c>
-      <c r="F24" s="42">
-        <v>2000000</v>
-      </c>
-      <c r="G24" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="H24" s="24">
-        <f>F24*12</f>
-        <v>24000000</v>
-      </c>
-      <c r="I24" s="24">
-        <f>H24*1.03</f>
-        <v>24720000</v>
-      </c>
-      <c r="J24" s="24">
-        <f t="shared" ref="J24:K24" si="1">I24*1.03</f>
-        <v>25461600</v>
-      </c>
-      <c r="K24" s="24">
-        <f t="shared" si="1"/>
-        <v>26225448</v>
-      </c>
-      <c r="L24" s="24">
-        <f>K24*1.03</f>
-        <v>27012211.440000001</v>
-      </c>
+      <c r="C24" s="28"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="23"/>
+      <c r="I24" s="23"/>
+      <c r="J24" s="23"/>
+      <c r="K24" s="23"/>
+      <c r="L24" s="23"/>
       <c r="M24" s="11"/>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B25" s="10"/>
-      <c r="C25" s="30"/>
+      <c r="C25" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" t="s">
+        <v>40</v>
+      </c>
       <c r="E25" t="s">
-        <v>37</v>
-      </c>
-      <c r="F25" s="42">
-        <v>500000</v>
+        <v>43</v>
+      </c>
+      <c r="F25" s="43">
+        <v>1000000</v>
       </c>
       <c r="G25" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="H25" s="24">
+      <c r="H25" s="23">
         <f>F25*12</f>
-        <v>6000000</v>
-      </c>
-      <c r="I25" s="24">
+        <v>12000000</v>
+      </c>
+      <c r="I25" s="23">
         <f>H25*1.03</f>
-        <v>6180000</v>
-      </c>
-      <c r="J25" s="24">
-        <f t="shared" ref="J25" si="2">I25*1.03</f>
-        <v>6365400</v>
-      </c>
-      <c r="K25" s="24">
-        <f t="shared" ref="K25" si="3">J25*1.03</f>
-        <v>6556362</v>
-      </c>
-      <c r="L25" s="24">
+        <v>12360000</v>
+      </c>
+      <c r="J25" s="23">
+        <f t="shared" ref="J25:K25" si="1">I25*1.03</f>
+        <v>12730800</v>
+      </c>
+      <c r="K25" s="23">
+        <f t="shared" si="1"/>
+        <v>13112724</v>
+      </c>
+      <c r="L25" s="23">
         <f>K25*1.03</f>
-        <v>6753052.8600000003</v>
+        <v>13506105.720000001</v>
       </c>
       <c r="M25" s="11"/>
     </row>
     <row r="26" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B26" s="10"/>
-      <c r="C26" s="30"/>
+      <c r="C26" s="28"/>
       <c r="E26" t="s">
+        <v>37</v>
+      </c>
+      <c r="F26" s="43">
+        <v>500000</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="H26" s="23">
+        <f>F26*12</f>
+        <v>6000000</v>
+      </c>
+      <c r="I26" s="23">
+        <f>H26*1.03</f>
+        <v>6180000</v>
+      </c>
+      <c r="J26" s="23">
+        <f t="shared" ref="J26" si="2">I26*1.03</f>
+        <v>6365400</v>
+      </c>
+      <c r="K26" s="23">
+        <f t="shared" ref="K26" si="3">J26*1.03</f>
+        <v>6556362</v>
+      </c>
+      <c r="L26" s="23">
+        <f>K26*1.03</f>
+        <v>6753052.8600000003</v>
+      </c>
+      <c r="M26" s="11"/>
+    </row>
+    <row r="27" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B27" s="10"/>
+      <c r="C27" s="28"/>
+      <c r="E27" t="s">
         <v>28</v>
       </c>
-      <c r="F26" s="42">
+      <c r="F27" s="43">
         <v>3000000</v>
       </c>
-      <c r="G26" s="12" t="s">
+      <c r="G27" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="H26" s="24">
-        <f>F26*14+F26*(4.75%+4.067%+1.15%)*14+F26</f>
+      <c r="H27" s="23">
+        <f>F27*14+F27*(4.75%+4.067%+1.15%)*14+F27</f>
         <v>49186140</v>
       </c>
-      <c r="I26" s="24">
-        <f>H26*1.03</f>
+      <c r="I27" s="23">
+        <f>H27*1.03</f>
         <v>50661724.200000003</v>
       </c>
-      <c r="J26" s="24">
-        <f t="shared" ref="J26:L26" si="4">I26*1.03</f>
+      <c r="J27" s="23">
+        <f t="shared" ref="J27:L27" si="4">I27*1.03</f>
         <v>52181575.926000006</v>
       </c>
-      <c r="K26" s="24">
+      <c r="K27" s="23">
         <f t="shared" si="4"/>
         <v>53747023.20378001</v>
       </c>
-      <c r="L26" s="24">
+      <c r="L27" s="23">
         <f t="shared" si="4"/>
         <v>55359433.899893411</v>
       </c>
-      <c r="M26" s="11"/>
-    </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B27" s="10"/>
-      <c r="C27" s="30"/>
-      <c r="E27" t="s">
+      <c r="M27" s="11"/>
+    </row>
+    <row r="28" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B28" s="10"/>
+      <c r="C28" s="28"/>
+      <c r="E28" t="s">
         <v>29</v>
       </c>
-      <c r="F27" s="42">
+      <c r="F28" s="43">
         <v>2000000</v>
       </c>
-      <c r="G27" s="12" t="s">
+      <c r="G28" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="H27" s="24">
-        <f t="shared" ref="H27:H29" si="5">F27*14+F27*(4.75%+4.067%+1.15%)*14+F27</f>
+      <c r="H28" s="23">
+        <f t="shared" ref="H28:H30" si="5">F28*14+F28*(4.75%+4.067%+1.15%)*14+F28</f>
         <v>32790760</v>
       </c>
-      <c r="I27" s="24">
-        <f t="shared" ref="I27:L27" si="6">H27*1.03</f>
+      <c r="I28" s="23">
+        <f t="shared" ref="I28:L28" si="6">H28*1.03</f>
         <v>33774482.800000004</v>
       </c>
-      <c r="J27" s="24">
+      <c r="J28" s="23">
         <f t="shared" si="6"/>
         <v>34787717.284000002</v>
       </c>
-      <c r="K27" s="24">
+      <c r="K28" s="23">
         <f t="shared" si="6"/>
         <v>35831348.802519999</v>
       </c>
-      <c r="L27" s="24">
+      <c r="L28" s="23">
         <f t="shared" si="6"/>
         <v>36906289.266595602</v>
       </c>
-      <c r="M27" s="11"/>
-    </row>
-    <row r="28" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B28" s="10"/>
-      <c r="C28" s="30"/>
-      <c r="E28" t="s">
+      <c r="M28" s="11"/>
+    </row>
+    <row r="29" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B29" s="10"/>
+      <c r="C29" s="28"/>
+      <c r="E29" t="s">
         <v>30</v>
       </c>
-      <c r="F28" s="42">
+      <c r="F29" s="43">
         <v>0</v>
       </c>
-      <c r="G28" s="12" t="s">
+      <c r="G29" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="H28" s="24">
+      <c r="H29" s="23">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I28" s="24">
-        <f t="shared" ref="I28:L28" si="7">H28*1.03</f>
+      <c r="I29" s="23">
+        <f t="shared" ref="I29:L29" si="7">H29*1.03</f>
         <v>0</v>
       </c>
-      <c r="J28" s="24">
+      <c r="J29" s="23">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="K28" s="24">
+      <c r="K29" s="23">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="L28" s="24">
+      <c r="L29" s="23">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="M28" s="11"/>
-    </row>
-    <row r="29" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B29" s="10"/>
-      <c r="C29" s="30"/>
-      <c r="E29" t="s">
+      <c r="M29" s="11"/>
+    </row>
+    <row r="30" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B30" s="10"/>
+      <c r="C30" s="28"/>
+      <c r="E30" t="s">
         <v>31</v>
       </c>
-      <c r="F29" s="42">
+      <c r="F30" s="43">
         <v>0</v>
       </c>
-      <c r="G29" s="12" t="s">
+      <c r="G30" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="H29" s="24">
+      <c r="H30" s="23">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I29" s="24">
-        <f t="shared" ref="I29:L30" si="8">H29*1.03</f>
+      <c r="I30" s="23">
+        <f t="shared" ref="I30:L31" si="8">H30*1.03</f>
         <v>0</v>
       </c>
-      <c r="J29" s="24">
+      <c r="J30" s="23">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="K29" s="24">
+      <c r="K30" s="23">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="L29" s="24">
+      <c r="L30" s="23">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="M29" s="11"/>
-    </row>
-    <row r="30" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B30" s="10"/>
-      <c r="C30" s="30"/>
-      <c r="E30" t="s">
+      <c r="M30" s="11"/>
+    </row>
+    <row r="31" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B31" s="10"/>
+      <c r="C31" s="28"/>
+      <c r="E31" t="s">
         <v>44</v>
       </c>
-      <c r="F30" s="42">
+      <c r="F31" s="43">
         <v>300000</v>
       </c>
-      <c r="G30" s="12" t="s">
+      <c r="G31" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="H30" s="24">
-        <f>F30*12</f>
+      <c r="H31" s="23">
+        <f>F31*12</f>
         <v>3600000</v>
       </c>
-      <c r="I30" s="24">
-        <f>H30*1.03</f>
+      <c r="I31" s="23">
+        <f>H31*1.03</f>
         <v>3708000</v>
       </c>
-      <c r="J30" s="24">
+      <c r="J31" s="23">
         <f t="shared" si="8"/>
         <v>3819240</v>
       </c>
-      <c r="K30" s="24">
+      <c r="K31" s="23">
         <f t="shared" si="8"/>
         <v>3933817.2</v>
       </c>
-      <c r="L30" s="24">
-        <f>K30*1.03</f>
+      <c r="L31" s="23">
+        <f>K31*1.03</f>
         <v>4051831.7160000005</v>
       </c>
-      <c r="M30" s="11"/>
-    </row>
-    <row r="31" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B31" s="10"/>
-      <c r="C31" s="30"/>
-      <c r="E31" t="s">
+      <c r="M31" s="11"/>
+    </row>
+    <row r="32" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B32" s="10"/>
+      <c r="C32" s="28"/>
+      <c r="E32" t="s">
         <v>18</v>
       </c>
-      <c r="F31" s="43">
+      <c r="F32" s="47">
         <v>0.05</v>
       </c>
-      <c r="G31" s="12" t="s">
+      <c r="G32" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="H31" s="24">
-        <f>H21*$F$31</f>
+      <c r="H32" s="23">
+        <f>H22*$F$32</f>
         <v>2760000</v>
       </c>
-      <c r="I31" s="24">
-        <f t="shared" ref="I31:L31" si="9">I21*$F$31</f>
+      <c r="I32" s="23">
+        <f t="shared" ref="I32:L32" si="9">I22*$F$32</f>
         <v>13800000</v>
       </c>
-      <c r="J31" s="24">
+      <c r="J32" s="23">
+        <f t="shared" si="9"/>
+        <v>16559999.999999998</v>
+      </c>
+      <c r="K32" s="23">
         <f t="shared" si="9"/>
         <v>19319999.999999996</v>
       </c>
-      <c r="K31" s="24">
+      <c r="L32" s="23">
         <f t="shared" si="9"/>
         <v>22080000</v>
       </c>
-      <c r="L31" s="24">
-        <f t="shared" si="9"/>
-        <v>24840000</v>
-      </c>
-      <c r="M31" s="11"/>
-    </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B32" s="10"/>
-      <c r="C32" s="30"/>
-      <c r="D32" s="36"/>
-      <c r="E32" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F32" s="44">
+      <c r="M32" s="11"/>
+    </row>
+    <row r="33" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B33" s="10"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="34"/>
+      <c r="E33" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F33" s="46">
         <v>200000</v>
       </c>
-      <c r="G32" s="4" t="s">
+      <c r="G33" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="H32" s="25">
-        <f>$F$32*12</f>
+      <c r="H33" s="24">
+        <f>$F$33*12</f>
         <v>2400000</v>
       </c>
-      <c r="I32" s="25">
-        <f t="shared" ref="I32:L32" si="10">$F$32*12</f>
+      <c r="I33" s="24">
+        <f t="shared" ref="I33:L33" si="10">$F$33*12</f>
         <v>2400000</v>
       </c>
-      <c r="J32" s="25">
+      <c r="J33" s="24">
         <f t="shared" si="10"/>
         <v>2400000</v>
       </c>
-      <c r="K32" s="25">
+      <c r="K33" s="24">
         <f t="shared" si="10"/>
         <v>2400000</v>
       </c>
-      <c r="L32" s="25">
+      <c r="L33" s="24">
         <f t="shared" si="10"/>
         <v>2400000</v>
       </c>
-      <c r="M32" s="11"/>
-    </row>
-    <row r="33" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B33" s="10"/>
-      <c r="C33" s="30"/>
-      <c r="E33" t="s">
-        <v>10</v>
-      </c>
-      <c r="F33" s="14">
-        <f>SUM(F24:F32)</f>
-        <v>8000000.0499999998</v>
-      </c>
-      <c r="G33" s="12"/>
-      <c r="H33" s="24">
-        <f>SUM(H24:H32)</f>
-        <v>120736900</v>
-      </c>
-      <c r="I33" s="24">
-        <f>SUM(I24:I32)</f>
-        <v>135244207</v>
-      </c>
-      <c r="J33" s="24">
-        <f>SUM(J24:J32)</f>
-        <v>144335533.21000001</v>
-      </c>
-      <c r="K33" s="24">
-        <f>SUM(K24:K32)</f>
-        <v>150773999.20630002</v>
-      </c>
-      <c r="L33" s="24">
-        <f>SUM(L24:L32)</f>
-        <v>157322819.18248904</v>
-      </c>
       <c r="M33" s="11"/>
     </row>
     <row r="34" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B34" s="10"/>
-      <c r="C34" s="30"/>
-      <c r="F34" s="14"/>
+      <c r="C34" s="28"/>
+      <c r="E34" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" s="14">
+        <f>SUM(F25:F33)</f>
+        <v>7000000.0499999998</v>
+      </c>
       <c r="G34" s="12"/>
-      <c r="H34" s="24"/>
-      <c r="I34" s="24"/>
-      <c r="J34" s="24"/>
-      <c r="K34" s="24"/>
-      <c r="L34" s="24"/>
+      <c r="H34" s="23">
+        <f>SUM(H25:H33)</f>
+        <v>108736900</v>
+      </c>
+      <c r="I34" s="23">
+        <f>SUM(I25:I33)</f>
+        <v>122884207</v>
+      </c>
+      <c r="J34" s="23">
+        <f>SUM(J25:J33)</f>
+        <v>128844733.21000001</v>
+      </c>
+      <c r="K34" s="23">
+        <f>SUM(K25:K33)</f>
+        <v>134901275.20630002</v>
+      </c>
+      <c r="L34" s="23">
+        <f>SUM(L25:L33)</f>
+        <v>141056713.46248901</v>
+      </c>
       <c r="M34" s="11"/>
     </row>
     <row r="35" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B35" s="10"/>
-      <c r="C35" s="30"/>
-      <c r="D35" t="s">
-        <v>52</v>
-      </c>
+      <c r="C35" s="28"/>
       <c r="F35" s="14"/>
       <c r="G35" s="12"/>
-      <c r="H35" s="24"/>
-      <c r="I35" s="24"/>
-      <c r="J35" s="24"/>
-      <c r="K35" s="24"/>
-      <c r="L35" s="24"/>
+      <c r="H35" s="23"/>
+      <c r="I35" s="23"/>
+      <c r="J35" s="23"/>
+      <c r="K35" s="23"/>
+      <c r="L35" s="23"/>
       <c r="M35" s="11"/>
     </row>
     <row r="36" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B36" s="10"/>
-      <c r="C36" s="30"/>
+      <c r="C36" s="28"/>
       <c r="D36" t="s">
-        <v>32</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="F36" s="14"/>
       <c r="G36" s="12"/>
-      <c r="H36" s="24"/>
-      <c r="I36" s="24"/>
-      <c r="J36" s="24"/>
-      <c r="K36" s="24"/>
-      <c r="L36" s="24"/>
+      <c r="H36" s="23"/>
+      <c r="I36" s="23"/>
+      <c r="J36" s="23"/>
+      <c r="K36" s="23"/>
+      <c r="L36" s="23"/>
       <c r="M36" s="11"/>
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B37" s="10"/>
-      <c r="C37" s="30"/>
+      <c r="C37" s="28"/>
+      <c r="D37" t="s">
+        <v>32</v>
+      </c>
       <c r="G37" s="12"/>
-      <c r="H37" s="24"/>
-      <c r="I37" s="24"/>
-      <c r="J37" s="24"/>
-      <c r="K37" s="24"/>
-      <c r="L37" s="24"/>
+      <c r="H37" s="23"/>
+      <c r="I37" s="23"/>
+      <c r="J37" s="23"/>
+      <c r="K37" s="23"/>
+      <c r="L37" s="23"/>
       <c r="M37" s="11"/>
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B38" s="10"/>
-      <c r="C38" s="30"/>
-      <c r="D38" t="s">
-        <v>41</v>
-      </c>
-      <c r="E38" t="s">
-        <v>2</v>
-      </c>
-      <c r="F38" s="43">
-        <v>0.4</v>
-      </c>
-      <c r="G38" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="H38" s="24">
-        <f>H21*$F$38</f>
-        <v>22080000</v>
-      </c>
-      <c r="I38" s="24">
-        <f>I21*$F$38</f>
-        <v>110400000</v>
-      </c>
-      <c r="J38" s="24">
-        <f>J21*$F$38</f>
-        <v>154559999.99999997</v>
-      </c>
-      <c r="K38" s="24">
-        <f>K21*$F$38</f>
-        <v>176640000</v>
-      </c>
-      <c r="L38" s="24">
-        <f>L21*$F$38</f>
-        <v>198720000</v>
-      </c>
+      <c r="C38" s="28"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="23"/>
+      <c r="I38" s="23"/>
+      <c r="J38" s="23"/>
+      <c r="K38" s="23"/>
+      <c r="L38" s="23"/>
       <c r="M38" s="11"/>
     </row>
     <row r="39" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B39" s="10"/>
-      <c r="C39" s="30"/>
+      <c r="C39" s="28"/>
+      <c r="D39" t="s">
+        <v>41</v>
+      </c>
       <c r="E39" t="s">
-        <v>5</v>
-      </c>
-      <c r="F39" s="43">
-        <v>0.06</v>
+        <v>2</v>
+      </c>
+      <c r="F39" s="47">
+        <v>0.4</v>
       </c>
       <c r="G39" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="H39" s="24">
-        <f>H21*$F$39</f>
-        <v>3312000</v>
-      </c>
-      <c r="I39" s="24">
-        <f>I21*$F$39</f>
-        <v>16560000</v>
-      </c>
-      <c r="J39" s="24">
-        <f>J21*$F$39</f>
-        <v>23183999.999999996</v>
-      </c>
-      <c r="K39" s="24">
-        <f>K21*$F$39</f>
-        <v>26496000</v>
-      </c>
-      <c r="L39" s="24">
-        <f>L21*$F$39</f>
-        <v>29808000</v>
+      <c r="H39" s="23">
+        <f>H22*$F$39</f>
+        <v>22080000</v>
+      </c>
+      <c r="I39" s="23">
+        <f>I22*$F$39</f>
+        <v>110400000</v>
+      </c>
+      <c r="J39" s="23">
+        <f>J22*$F$39</f>
+        <v>132479999.99999999</v>
+      </c>
+      <c r="K39" s="23">
+        <f>K22*$F$39</f>
+        <v>154559999.99999997</v>
+      </c>
+      <c r="L39" s="23">
+        <f>L22*$F$39</f>
+        <v>176640000</v>
       </c>
       <c r="M39" s="11"/>
     </row>
     <row r="40" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B40" s="10"/>
-      <c r="C40" s="30"/>
+      <c r="C40" s="28"/>
       <c r="E40" t="s">
-        <v>6</v>
-      </c>
-      <c r="F40" s="43">
+        <v>5</v>
+      </c>
+      <c r="F40" s="47">
         <v>0.05</v>
       </c>
       <c r="G40" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="H40" s="24">
-        <f>H21*$F$40</f>
+      <c r="H40" s="23">
+        <f>H22*$F$40</f>
         <v>2760000</v>
       </c>
-      <c r="I40" s="24">
-        <f>I21*$F$40</f>
+      <c r="I40" s="23">
+        <f>I22*$F$40</f>
         <v>13800000</v>
       </c>
-      <c r="J40" s="24">
-        <f>J21*$F$40</f>
+      <c r="J40" s="23">
+        <f>J22*$F$40</f>
+        <v>16559999.999999998</v>
+      </c>
+      <c r="K40" s="23">
+        <f>K22*$F$40</f>
         <v>19319999.999999996</v>
       </c>
-      <c r="K40" s="24">
-        <f>K21*$F$40</f>
+      <c r="L40" s="23">
+        <f>L22*$F$40</f>
         <v>22080000</v>
-      </c>
-      <c r="L40" s="24">
-        <f>L21*$F$40</f>
-        <v>24840000</v>
       </c>
       <c r="M40" s="11"/>
     </row>
     <row r="41" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B41" s="10"/>
-      <c r="C41" s="30"/>
+      <c r="C41" s="28"/>
       <c r="E41" t="s">
-        <v>21</v>
-      </c>
-      <c r="F41" s="43">
-        <v>0.03</v>
+        <v>6</v>
+      </c>
+      <c r="F41" s="47">
+        <v>0.04</v>
       </c>
       <c r="G41" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="H41" s="24">
-        <f>H21*$F$41</f>
-        <v>1656000</v>
-      </c>
-      <c r="I41" s="24">
-        <f>I21*$F$41</f>
-        <v>8280000</v>
-      </c>
-      <c r="J41" s="24">
-        <f>J21*$F$41</f>
-        <v>11591999.999999998</v>
-      </c>
-      <c r="K41" s="24">
-        <f>K21*$F$41</f>
-        <v>13248000</v>
-      </c>
-      <c r="L41" s="24">
-        <f>L21*$F$41</f>
-        <v>14904000</v>
+      <c r="H41" s="23">
+        <f>H22*$F$41</f>
+        <v>2208000</v>
+      </c>
+      <c r="I41" s="23">
+        <f>I22*$F$41</f>
+        <v>11040000</v>
+      </c>
+      <c r="J41" s="23">
+        <f>J22*$F$41</f>
+        <v>13247999.999999998</v>
+      </c>
+      <c r="K41" s="23">
+        <f>K22*$F$41</f>
+        <v>15455999.999999998</v>
+      </c>
+      <c r="L41" s="23">
+        <f>L22*$F$41</f>
+        <v>17664000</v>
       </c>
       <c r="M41" s="11"/>
     </row>
     <row r="42" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B42" s="10"/>
-      <c r="C42" s="30"/>
+      <c r="C42" s="28"/>
       <c r="E42" t="s">
-        <v>38</v>
-      </c>
-      <c r="F42" s="43">
-        <v>0.01</v>
+        <v>21</v>
+      </c>
+      <c r="F42" s="47">
+        <v>0.03</v>
       </c>
       <c r="G42" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="H42" s="24">
-        <f>H21*$F$42</f>
-        <v>552000</v>
-      </c>
-      <c r="I42" s="24">
-        <f>I21*$F$42</f>
-        <v>2760000</v>
-      </c>
-      <c r="J42" s="24">
-        <f>J21*$F$42</f>
-        <v>3863999.9999999995</v>
-      </c>
-      <c r="K42" s="24">
-        <f>K21*$F$42</f>
-        <v>4416000</v>
-      </c>
-      <c r="L42" s="24">
-        <f>L21*$F$42</f>
-        <v>4968000</v>
+      <c r="H42" s="23">
+        <f>H22*$F$42</f>
+        <v>1656000</v>
+      </c>
+      <c r="I42" s="23">
+        <f>I22*$F$42</f>
+        <v>8280000</v>
+      </c>
+      <c r="J42" s="23">
+        <f>J22*$F$42</f>
+        <v>9935999.9999999981</v>
+      </c>
+      <c r="K42" s="23">
+        <f>K22*$F$42</f>
+        <v>11591999.999999998</v>
+      </c>
+      <c r="L42" s="23">
+        <f>L22*$F$42</f>
+        <v>13248000</v>
       </c>
       <c r="M42" s="11"/>
     </row>
     <row r="43" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B43" s="10"/>
-      <c r="C43" s="30"/>
-      <c r="D43" s="36"/>
-      <c r="E43" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F43" s="39">
+      <c r="C43" s="28"/>
+      <c r="E43" t="s">
+        <v>38</v>
+      </c>
+      <c r="F43" s="47">
+        <v>0.01</v>
+      </c>
+      <c r="G43" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="H43" s="23">
+        <f>H22*$F$43</f>
+        <v>552000</v>
+      </c>
+      <c r="I43" s="23">
+        <f>I22*$F$43</f>
+        <v>2760000</v>
+      </c>
+      <c r="J43" s="23">
+        <f>J22*$F$43</f>
+        <v>3311999.9999999995</v>
+      </c>
+      <c r="K43" s="23">
+        <f>K22*$F$43</f>
+        <v>3863999.9999999995</v>
+      </c>
+      <c r="L43" s="23">
+        <f>L22*$F$43</f>
+        <v>4416000</v>
+      </c>
+      <c r="M43" s="11"/>
+    </row>
+    <row r="44" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B44" s="10"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="34"/>
+      <c r="E44" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F44" s="37">
         <v>0.08</v>
       </c>
-      <c r="G43" s="4"/>
-      <c r="H43" s="25">
-        <f>H21*$F$43</f>
+      <c r="G44" s="4"/>
+      <c r="H44" s="24">
+        <f>H22*$F$44</f>
         <v>4416000</v>
       </c>
-      <c r="I43" s="25">
-        <f t="shared" ref="I43:L43" si="11">I21*$F$43</f>
+      <c r="I44" s="24">
+        <f t="shared" ref="I44:L44" si="11">I22*$F$44</f>
         <v>22080000</v>
       </c>
-      <c r="J43" s="25">
+      <c r="J44" s="24">
+        <f t="shared" si="11"/>
+        <v>26495999.999999996</v>
+      </c>
+      <c r="K44" s="24">
         <f t="shared" si="11"/>
         <v>30911999.999999996</v>
       </c>
-      <c r="K43" s="25">
+      <c r="L44" s="24">
         <f t="shared" si="11"/>
         <v>35328000</v>
       </c>
-      <c r="L43" s="25">
-        <f t="shared" si="11"/>
-        <v>39744000</v>
-      </c>
-      <c r="M43" s="11"/>
-    </row>
-    <row r="44" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B44" s="10"/>
-      <c r="C44" s="30"/>
-      <c r="E44" t="s">
-        <v>10</v>
-      </c>
-      <c r="F44" s="15">
-        <f>SUM(F38:F43)</f>
-        <v>0.63</v>
-      </c>
-      <c r="G44" s="12"/>
-      <c r="H44" s="24">
-        <f>SUM(H38:H43)</f>
-        <v>34776000</v>
-      </c>
-      <c r="I44" s="24">
-        <f>SUM(I38:I43)</f>
-        <v>173880000</v>
-      </c>
-      <c r="J44" s="24">
-        <f>SUM(J38:J43)</f>
-        <v>243431999.99999997</v>
-      </c>
-      <c r="K44" s="24">
-        <f>SUM(K38:K43)</f>
-        <v>278208000</v>
-      </c>
-      <c r="L44" s="24">
-        <f>SUM(L38:L43)</f>
-        <v>312984000</v>
-      </c>
       <c r="M44" s="11"/>
     </row>
     <row r="45" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B45" s="10"/>
-      <c r="C45" s="30"/>
+      <c r="C45" s="28"/>
+      <c r="E45" t="s">
+        <v>10</v>
+      </c>
+      <c r="F45" s="15">
+        <f>SUM(F39:F44)</f>
+        <v>0.61</v>
+      </c>
       <c r="G45" s="12"/>
-      <c r="H45" s="24"/>
-      <c r="I45" s="24"/>
-      <c r="J45" s="24"/>
-      <c r="K45" s="24"/>
-      <c r="L45" s="24"/>
+      <c r="H45" s="23">
+        <f>SUM(H39:H44)</f>
+        <v>33672000</v>
+      </c>
+      <c r="I45" s="23">
+        <f>SUM(I39:I44)</f>
+        <v>168360000</v>
+      </c>
+      <c r="J45" s="23">
+        <f>SUM(J39:J44)</f>
+        <v>202031999.99999997</v>
+      </c>
+      <c r="K45" s="23">
+        <f>SUM(K39:K44)</f>
+        <v>235703999.99999997</v>
+      </c>
+      <c r="L45" s="23">
+        <f>SUM(L39:L44)</f>
+        <v>269376000</v>
+      </c>
       <c r="M45" s="11"/>
     </row>
     <row r="46" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B46" s="10"/>
-      <c r="C46" s="30"/>
+      <c r="C46" s="28"/>
       <c r="G46" s="12"/>
-      <c r="H46" s="24"/>
-      <c r="I46" s="24"/>
-      <c r="J46" s="24"/>
-      <c r="K46" s="24"/>
-      <c r="L46" s="24"/>
+      <c r="H46" s="23"/>
+      <c r="I46" s="23"/>
+      <c r="J46" s="23"/>
+      <c r="K46" s="23"/>
+      <c r="L46" s="23"/>
       <c r="M46" s="11"/>
     </row>
     <row r="47" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B47" s="10"/>
-      <c r="C47" s="30"/>
-      <c r="D47" t="s">
-        <v>42</v>
-      </c>
+      <c r="C47" s="28"/>
       <c r="G47" s="12"/>
-      <c r="H47" s="24">
-        <f>H33+H44</f>
-        <v>155512900</v>
-      </c>
-      <c r="I47" s="24">
-        <f>I33+I44</f>
-        <v>309124207</v>
-      </c>
-      <c r="J47" s="24">
-        <f>J33+J44</f>
-        <v>387767533.20999998</v>
-      </c>
-      <c r="K47" s="24">
-        <f>K33+K44</f>
-        <v>428981999.20630002</v>
-      </c>
-      <c r="L47" s="24">
-        <f>L33+L44</f>
-        <v>470306819.18248904</v>
-      </c>
+      <c r="H47" s="23"/>
+      <c r="I47" s="23"/>
+      <c r="J47" s="23"/>
+      <c r="K47" s="23"/>
+      <c r="L47" s="23"/>
       <c r="M47" s="11"/>
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B48" s="10"/>
-      <c r="C48" s="30"/>
-      <c r="H48" s="26"/>
-      <c r="I48" s="26"/>
-      <c r="J48" s="26"/>
-      <c r="K48" s="26"/>
-      <c r="L48" s="26"/>
+      <c r="C48" s="28"/>
+      <c r="D48" t="s">
+        <v>42</v>
+      </c>
+      <c r="G48" s="12"/>
+      <c r="H48" s="23">
+        <f>H34+H45</f>
+        <v>142408900</v>
+      </c>
+      <c r="I48" s="23">
+        <f>I34+I45</f>
+        <v>291244207</v>
+      </c>
+      <c r="J48" s="23">
+        <f>J34+J45</f>
+        <v>330876733.20999998</v>
+      </c>
+      <c r="K48" s="23">
+        <f>K34+K45</f>
+        <v>370605275.20630002</v>
+      </c>
+      <c r="L48" s="23">
+        <f>L34+L45</f>
+        <v>410432713.46248901</v>
+      </c>
       <c r="M48" s="11"/>
     </row>
     <row r="49" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B49" s="10"/>
-      <c r="C49" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="D49" s="16"/>
-      <c r="E49" s="16"/>
-      <c r="F49" s="17"/>
-      <c r="G49" s="46">
-        <f t="shared" ref="G49:L49" si="12">G21-G47-G18</f>
-        <v>-30000000</v>
-      </c>
-      <c r="H49" s="46">
-        <f t="shared" si="12"/>
-        <v>-100312900</v>
-      </c>
-      <c r="I49" s="46">
-        <f t="shared" si="12"/>
-        <v>-33124207</v>
-      </c>
-      <c r="J49" s="46">
-        <f t="shared" si="12"/>
-        <v>-1367533.2100000381</v>
-      </c>
-      <c r="K49" s="46">
-        <f t="shared" si="12"/>
-        <v>12618000.79369998</v>
-      </c>
-      <c r="L49" s="46">
-        <f t="shared" si="12"/>
-        <v>26493180.817510962</v>
-      </c>
+      <c r="C49" s="28"/>
+      <c r="H49" s="25"/>
+      <c r="I49" s="25"/>
+      <c r="J49" s="25"/>
+      <c r="K49" s="25"/>
+      <c r="L49" s="25"/>
       <c r="M49" s="11"/>
     </row>
     <row r="50" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B50" s="10"/>
-      <c r="C50" s="30"/>
-      <c r="E50" t="s">
-        <v>19</v>
-      </c>
-      <c r="G50" s="18">
-        <f>G49</f>
-        <v>-30000000</v>
-      </c>
-      <c r="H50" s="27">
-        <f>G50+H49</f>
-        <v>-130312900</v>
-      </c>
-      <c r="I50" s="27">
-        <f>H50+I49</f>
-        <v>-163437107</v>
-      </c>
-      <c r="J50" s="27">
-        <f t="shared" ref="J50:L50" si="13">I50+J49</f>
-        <v>-164804640.21000004</v>
-      </c>
-      <c r="K50" s="27">
-        <f t="shared" si="13"/>
-        <v>-152186639.41630006</v>
-      </c>
-      <c r="L50" s="27">
-        <f t="shared" si="13"/>
-        <v>-125693458.5987891</v>
+      <c r="C50" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="D50" s="16"/>
+      <c r="E50" s="16"/>
+      <c r="F50" s="17"/>
+      <c r="G50" s="51"/>
+      <c r="H50" s="51">
+        <f>H22-H48</f>
+        <v>-87208900</v>
+      </c>
+      <c r="I50" s="51">
+        <f t="shared" ref="I50:L50" si="12">I22-I48</f>
+        <v>-15244207</v>
+      </c>
+      <c r="J50" s="51">
+        <f t="shared" si="12"/>
+        <v>323266.78999996185</v>
+      </c>
+      <c r="K50" s="51">
+        <f t="shared" si="12"/>
+        <v>15794724.79369992</v>
+      </c>
+      <c r="L50" s="51">
+        <f t="shared" si="12"/>
+        <v>31167286.537510991</v>
       </c>
       <c r="M50" s="11"/>
     </row>
     <row r="51" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B51" s="10"/>
-      <c r="C51" s="30"/>
-      <c r="H51" s="26"/>
-      <c r="I51" s="26"/>
-      <c r="J51" s="26"/>
-      <c r="K51" s="26"/>
-      <c r="L51" s="26"/>
+      <c r="C51" s="28"/>
+      <c r="E51" t="s">
+        <v>19</v>
+      </c>
+      <c r="G51" s="12"/>
+      <c r="H51" s="52">
+        <f>H50</f>
+        <v>-87208900</v>
+      </c>
+      <c r="I51" s="52">
+        <f>H51+I50</f>
+        <v>-102453107</v>
+      </c>
+      <c r="J51" s="52">
+        <f t="shared" ref="J51:L51" si="13">I51+J50</f>
+        <v>-102129840.21000004</v>
+      </c>
+      <c r="K51" s="52">
+        <f t="shared" si="13"/>
+        <v>-86335115.416300118</v>
+      </c>
+      <c r="L51" s="52">
+        <f t="shared" si="13"/>
+        <v>-55167828.878789127</v>
+      </c>
       <c r="M51" s="11"/>
     </row>
     <row r="52" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B52" s="10"/>
-      <c r="C52" s="31" t="s">
+      <c r="C52" s="28"/>
+      <c r="H52" s="25"/>
+      <c r="I52" s="25"/>
+      <c r="J52" s="25"/>
+      <c r="K52" s="25"/>
+      <c r="L52" s="25"/>
+      <c r="M52" s="11"/>
+    </row>
+    <row r="53" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B53" s="10"/>
+      <c r="C53" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="D52" s="16"/>
-      <c r="E52" s="16"/>
-      <c r="F52" s="17"/>
-      <c r="G52" s="34">
-        <f t="shared" ref="G52:L52" si="14">$G$11+G50</f>
-        <v>170000000</v>
-      </c>
-      <c r="H52" s="35">
+      <c r="D53" s="16"/>
+      <c r="E53" s="16"/>
+      <c r="F53" s="17"/>
+      <c r="G53" s="32">
+        <f>$G$11-G19</f>
+        <v>160000000</v>
+      </c>
+      <c r="H53" s="33">
+        <f>G53+H50</f>
+        <v>72791100</v>
+      </c>
+      <c r="I53" s="33">
+        <f t="shared" ref="I53:L53" si="14">H53+I50</f>
+        <v>57546893</v>
+      </c>
+      <c r="J53" s="33">
         <f t="shared" si="14"/>
-        <v>69687100</v>
-      </c>
-      <c r="I52" s="35">
+        <v>57870159.789999962</v>
+      </c>
+      <c r="K53" s="33">
         <f t="shared" si="14"/>
-        <v>36562893</v>
-      </c>
-      <c r="J52" s="35">
+        <v>73664884.583699882</v>
+      </c>
+      <c r="L53" s="33">
         <f t="shared" si="14"/>
-        <v>35195359.789999962</v>
-      </c>
-      <c r="K52" s="35">
-        <f t="shared" si="14"/>
-        <v>47813360.583699942</v>
-      </c>
-      <c r="L52" s="35">
-        <f t="shared" si="14"/>
-        <v>74306541.401210904</v>
-      </c>
-      <c r="M52" s="11"/>
-    </row>
-    <row r="53" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B53" s="19"/>
-      <c r="C53" s="32"/>
-      <c r="D53" s="20"/>
-      <c r="E53" s="20"/>
-      <c r="F53" s="21"/>
-      <c r="G53" s="20"/>
-      <c r="H53" s="28"/>
-      <c r="I53" s="28"/>
-      <c r="J53" s="28"/>
-      <c r="K53" s="28"/>
-      <c r="L53" s="28"/>
-      <c r="M53" s="22"/>
+        <v>104832171.12121087</v>
+      </c>
+      <c r="M53" s="11"/>
+    </row>
+    <row r="54" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B54" s="18"/>
+      <c r="C54" s="30"/>
+      <c r="D54" s="19"/>
+      <c r="E54" s="19"/>
+      <c r="F54" s="20"/>
+      <c r="G54" s="19"/>
+      <c r="H54" s="26"/>
+      <c r="I54" s="26"/>
+      <c r="J54" s="26"/>
+      <c r="K54" s="26"/>
+      <c r="L54" s="26"/>
+      <c r="M54" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>